<commit_message>
Update workflow.xlsx from Gmail job: Notification Test 1018
</commit_message>
<xml_diff>
--- a/workflow.xlsx
+++ b/workflow.xlsx
@@ -507,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R31"/>
+  <dimension ref="A1:R32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="11.6640625" customWidth="1" style="20" min="1" max="1"/>
@@ -1730,6 +1730,33 @@
       </c>
       <c r="L31" s="18" t="n"/>
       <c r="M31" s="18" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="22" t="n"/>
+      <c r="B32" s="17" t="n"/>
+      <c r="C32" s="17" t="n"/>
+      <c r="D32" s="17" t="n"/>
+      <c r="E32" s="17" t="n"/>
+      <c r="F32" s="17" t="n"/>
+      <c r="G32" s="17" t="inlineStr">
+        <is>
+          <t>TBI</t>
+        </is>
+      </c>
+      <c r="H32" s="17" t="inlineStr">
+        <is>
+          <t>Notification Test 1018</t>
+        </is>
+      </c>
+      <c r="I32" s="17" t="n"/>
+      <c r="J32" s="17" t="n"/>
+      <c r="K32" s="23" t="inlineStr">
+        <is>
+          <t>31-10-2026 04:04:52 PM</t>
+        </is>
+      </c>
+      <c r="L32" s="18" t="n"/>
+      <c r="M32" s="18" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update workflow.xlsx from Gmail job: Notification Test 1019
</commit_message>
<xml_diff>
--- a/workflow.xlsx
+++ b/workflow.xlsx
@@ -507,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R32"/>
+  <dimension ref="A1:R33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="11.6640625" customWidth="1" style="20" min="1" max="1"/>
@@ -1757,6 +1757,33 @@
       </c>
       <c r="L32" s="18" t="n"/>
       <c r="M32" s="18" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="22" t="n"/>
+      <c r="B33" s="17" t="n"/>
+      <c r="C33" s="17" t="n"/>
+      <c r="D33" s="17" t="n"/>
+      <c r="E33" s="17" t="n"/>
+      <c r="F33" s="17" t="n"/>
+      <c r="G33" s="17" t="inlineStr">
+        <is>
+          <t>TBI</t>
+        </is>
+      </c>
+      <c r="H33" s="17" t="inlineStr">
+        <is>
+          <t>Notification Test 1019</t>
+        </is>
+      </c>
+      <c r="I33" s="17" t="n"/>
+      <c r="J33" s="17" t="n"/>
+      <c r="K33" s="23" t="inlineStr">
+        <is>
+          <t>31-10-2026 05:09:13 PM</t>
+        </is>
+      </c>
+      <c r="L33" s="18" t="n"/>
+      <c r="M33" s="18" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>